<commit_message>
Fase 4: chequeo 2 como diagnostico, motion_check y signal_check arreglados, junto_al_borde
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_063_CTRL1_5V/contracciones.xlsx
+++ b/data/processed_data/Video_063_CTRL1_5V/contracciones.xlsx
@@ -24,16 +24,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,22 +424,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>k</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>umbral_px</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>eventos</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>falsos_control</t>
         </is>
@@ -790,321 +778,326 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK2"/>
+  <dimension ref="A1:BL2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>canal</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>n_frames</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>duracion_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>signo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ruido_canal_px</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ruido_grosor_px</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>n_eventos</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>k_usado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>k_automatico</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>hay_meseta</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>meseta_motivo</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>meseta_k_rango</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>conteo_reportable</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>intervalo_mediano_s</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>amplitud_traslacion_px</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>ritmo</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>fps_medido</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>adelgazamiento_px</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>adelgazamiento_sigma</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>retardo_adelgazamiento_s</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>cociente_adelg_trasl_pct</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>adelgazamiento_robusto_px</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>adelgazamiento_robusto_sigma</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>cociente_robusto_pct</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>blur_px</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>blur_sigma</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>cinetica_grupo_principal</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>n_eventos_cinetica</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>amplitud_relativa_iqr_pct</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>eventos_junto_al_borde</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
         </is>
@@ -1294,37 +1287,40 @@
         <v>0</v>
       </c>
       <c r="BB2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC2" t="n">
         <v>2</v>
       </c>
-      <c r="BC2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BD2" t="n">
+      <c r="BD2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BE2" t="n">
         <v>0.2333333333333201</v>
       </c>
-      <c r="BE2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="inlineStr">
+      <c r="BF2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="inlineStr">
         <is>
           <t>1.5 s: 6 | 2 s: 6 | 3 s: 6</t>
         </is>
       </c>
-      <c r="BG2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BH2" t="inlineStr">
+      <c r="BH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI2" t="inlineStr">
         <is>
           <t>6 ev en k=9.415-13.785; 5 ev en k=15.163-24.421</t>
         </is>
       </c>
-      <c r="BI2" t="n">
+      <c r="BJ2" t="n">
         <v>0.03513762000002872</v>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BK2" t="n">
         <v>0.03217241999984601</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BL2" t="n">
         <v>1.092165898623632</v>
       </c>
     </row>
@@ -1343,52 +1339,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>t_inicio_s</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>t_fin_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>intervalo_mediano_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>intervalo_IQR_s</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>frecuencia_mediana_Hz</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>CV_intervalo_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>amplitud_mediana_px</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>amplitud_IQR_px</t>
         </is>
@@ -1469,87 +1465,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tren</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>busqueda</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>veredicto</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>clasificacion</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>periodo_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>periodo_err_s</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>frecuencia_Hz</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>jitter_ms</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>z</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>p_valor</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>n_eventos_tren</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>n_ranuras</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>captura_pct</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>n_dudosos</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>n_sacados_tiempo_amplitud</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>inicio_s</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>fin_s</t>
         </is>
@@ -1629,32 +1625,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tren</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ranura</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>t_esperado_s</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>t_medido_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>error_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>capturada</t>
         </is>
@@ -1771,28 +1767,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>evento</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>tiempo_s</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>amplitud_px</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>junto_a_hueco</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>junto_al_borde</t>
         </is>
       </c>
     </row>
@@ -1808,6 +1809,9 @@
       </c>
       <c r="D2" t="b">
         <v>0</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1823,6 +1827,9 @@
       <c r="D3" t="b">
         <v>0</v>
       </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1837,6 +1844,9 @@
       <c r="D4" t="b">
         <v>0</v>
       </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1851,6 +1861,9 @@
       <c r="D5" t="b">
         <v>0</v>
       </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1865,6 +1878,9 @@
       <c r="D6" t="b">
         <v>0</v>
       </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1877,6 +1893,9 @@
         <v>1.588099999999997</v>
       </c>
       <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1895,117 +1914,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>evento</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>tren</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>frame_pico</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>tiempo_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>amplitud_px</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>grosor_reposo_px</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>meseta_pico_frames</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>onset_s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_frames</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_min_s</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ttp_max_s</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ttp_medible</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rt50_frames</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_min_s</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_max_s</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_medible</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>offset_s</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>duracion_frames</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>duracion_s</t>
         </is>
@@ -2464,112 +2483,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>n_eventos_cinetica</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>amplitud_relativa_iqr_pct</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>

</xml_diff>